<commit_message>
feat: implement backend services and frontend modules for villa management, billing, invoicing, and role-based access control.
</commit_message>
<xml_diff>
--- a/Community_Testing_Credentials.xlsx
+++ b/Community_Testing_Credentials.xlsx
@@ -429,7 +429,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Admin / Staff</v>
+        <v>Community Admin</v>
       </c>
       <c r="B2" t="str">
         <v>Community Admin</v>
@@ -507,7 +507,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Tenant</v>
+        <v>Resident Tenant</v>
       </c>
       <c r="B5" t="str">
         <v>Rahul Mehta (Tenant 1)</v>
@@ -533,7 +533,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tenant</v>
+        <v>Resident Tenant</v>
       </c>
       <c r="B6" t="str">
         <v>Aisha Khan (Tenant 2)</v>
@@ -750,7 +750,7 @@
         <v>SCEN-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Tenant (tenant1)</v>
+        <v>Resident Tenant (tenant1)</v>
       </c>
       <c r="C4" t="str">
         <v>Outstanding Balance &amp; Pay Now Trigger</v>

</xml_diff>

<commit_message>
chore(testing): regenerate community credentials and seed data
</commit_message>
<xml_diff>
--- a/Community_Testing_Credentials.xlsx
+++ b/Community_Testing_Credentials.xlsx
@@ -467,10 +467,10 @@
         <v>Super Admin</v>
       </c>
       <c r="E2" t="str">
-        <v>admin@enterprise.com</v>
+        <v>admin@managemygate.com</v>
       </c>
       <c r="F2" t="str">
-        <v>SuperAdminPwd@123</v>
+        <v>password123</v>
       </c>
       <c r="G2" t="str">
         <v>superadmin</v>
@@ -499,7 +499,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D3" t="str">
-        <v>Rohit Bose</v>
+        <v>Aarav Menon</v>
       </c>
       <c r="E3" t="str">
         <v>admin1@greenfield.com</v>
@@ -534,7 +534,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D4" t="str">
-        <v>Harish Kumar</v>
+        <v>Rohit Gupta</v>
       </c>
       <c r="E4" t="str">
         <v>admin2@greenfield.com</v>
@@ -569,7 +569,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D5" t="str">
-        <v>Sanjay Kapoor</v>
+        <v>Rajesh Banerjee</v>
       </c>
       <c r="E5" t="str">
         <v>fm1@greenfield.com</v>
@@ -604,7 +604,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D6" t="str">
-        <v>Zara Sharma</v>
+        <v>Aarav Joshi</v>
       </c>
       <c r="E6" t="str">
         <v>fm2@greenfield.com</v>
@@ -639,7 +639,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D7" t="str">
-        <v>Vikram Mehta</v>
+        <v>Tanvi Bhat</v>
       </c>
       <c r="E7" t="str">
         <v>guard1@greenfield.com</v>
@@ -674,7 +674,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D8" t="str">
-        <v>Siddharth Gupta</v>
+        <v>Arjun Singh</v>
       </c>
       <c r="E8" t="str">
         <v>guard2@greenfield.com</v>
@@ -709,7 +709,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Ishaan Sinha</v>
+        <v>Sanjay Sharma</v>
       </c>
       <c r="E9" t="str">
         <v>owner1@greenfield.com</v>
@@ -744,7 +744,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Bhavna Shah</v>
+        <v>Akash Iyer</v>
       </c>
       <c r="E10" t="str">
         <v>owner2@greenfield.com</v>
@@ -779,7 +779,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Aditi Ghosh</v>
+        <v>Arjun Desai</v>
       </c>
       <c r="E11" t="str">
         <v>owner3@greenfield.com</v>
@@ -814,7 +814,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Rajesh Mehta</v>
+        <v>Yamini Bose</v>
       </c>
       <c r="E12" t="str">
         <v>owner4@greenfield.com</v>
@@ -849,7 +849,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D13" t="str">
-        <v>Siddharth Iyer</v>
+        <v>Tanvi Iyer</v>
       </c>
       <c r="E13" t="str">
         <v>owner5@greenfield.com</v>
@@ -884,7 +884,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D14" t="str">
-        <v>Rahul Patel</v>
+        <v>Rekha Mishra</v>
       </c>
       <c r="E14" t="str">
         <v>owner6@greenfield.com</v>
@@ -919,7 +919,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D15" t="str">
-        <v>Priya Verma</v>
+        <v>Ananya Iyer</v>
       </c>
       <c r="E15" t="str">
         <v>owner7@greenfield.com</v>
@@ -954,7 +954,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D16" t="str">
-        <v>Tanvi Shah</v>
+        <v>Rahul Verma</v>
       </c>
       <c r="E16" t="str">
         <v>owner8@greenfield.com</v>
@@ -989,7 +989,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D17" t="str">
-        <v>Jaya Mehta</v>
+        <v>Sanjay Mehta</v>
       </c>
       <c r="E17" t="str">
         <v>owner9@greenfield.com</v>
@@ -1024,7 +1024,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D18" t="str">
-        <v>Sahil Kumar</v>
+        <v>Sahil Rao</v>
       </c>
       <c r="E18" t="str">
         <v>owner10@greenfield.com</v>
@@ -1059,7 +1059,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Siddharth Mehta</v>
+        <v>Om Banerjee</v>
       </c>
       <c r="E19" t="str">
         <v>tenant1@greenfield.com</v>
@@ -1094,7 +1094,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D20" t="str">
-        <v>Harish Banerjee</v>
+        <v>Aditi Agarwal</v>
       </c>
       <c r="E20" t="str">
         <v>tenant2@greenfield.com</v>
@@ -1129,7 +1129,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D21" t="str">
-        <v>Chirag Rao</v>
+        <v>Rajesh Pillai</v>
       </c>
       <c r="E21" t="str">
         <v>tenant3@greenfield.com</v>
@@ -1164,7 +1164,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D22" t="str">
-        <v>Yamini Gupta</v>
+        <v>Meera Patel</v>
       </c>
       <c r="E22" t="str">
         <v>tenant4@greenfield.com</v>
@@ -1199,7 +1199,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D23" t="str">
-        <v>Rajesh Banerjee</v>
+        <v>Vikram Singh</v>
       </c>
       <c r="E23" t="str">
         <v>tenant5@greenfield.com</v>
@@ -1234,7 +1234,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D24" t="str">
-        <v>Kavya Patel</v>
+        <v>Shiv Reddy</v>
       </c>
       <c r="E24" t="str">
         <v>tenant6@greenfield.com</v>
@@ -1269,7 +1269,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D25" t="str">
-        <v>Ananya Banerjee</v>
+        <v>Arjun Verma</v>
       </c>
       <c r="E25" t="str">
         <v>tenant7@greenfield.com</v>
@@ -1304,7 +1304,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D26" t="str">
-        <v>Vinay Banerjee</v>
+        <v>Priya Ghosh</v>
       </c>
       <c r="E26" t="str">
         <v>tenant8@greenfield.com</v>
@@ -1339,7 +1339,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D27" t="str">
-        <v>Divya Singh</v>
+        <v>Meera Mehta</v>
       </c>
       <c r="E27" t="str">
         <v>tenant9@greenfield.com</v>
@@ -1374,7 +1374,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D28" t="str">
-        <v>Kavya Bose</v>
+        <v>Jaya Kumar</v>
       </c>
       <c r="E28" t="str">
         <v>tenant10@greenfield.com</v>
@@ -1409,7 +1409,7 @@
         <v>Family Member</v>
       </c>
       <c r="D29" t="str">
-        <v>Farhan Pandey</v>
+        <v>Divya Bose</v>
       </c>
       <c r="E29" t="str">
         <v>family1@greenfield.com</v>
@@ -1444,7 +1444,7 @@
         <v>Family Member</v>
       </c>
       <c r="D30" t="str">
-        <v>Varun Ghosh</v>
+        <v>Ishaan Sharma</v>
       </c>
       <c r="E30" t="str">
         <v>family2@greenfield.com</v>
@@ -1479,7 +1479,7 @@
         <v>Family Member</v>
       </c>
       <c r="D31" t="str">
-        <v>Nisha Rao</v>
+        <v>Zara Verma</v>
       </c>
       <c r="E31" t="str">
         <v>family3@greenfield.com</v>
@@ -1514,7 +1514,7 @@
         <v>Family Member</v>
       </c>
       <c r="D32" t="str">
-        <v>Rajesh Nair</v>
+        <v>Chirag Bhat</v>
       </c>
       <c r="E32" t="str">
         <v>family4@greenfield.com</v>
@@ -1549,7 +1549,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D33" t="str">
-        <v>Varun Pandey</v>
+        <v>Karan Pillai</v>
       </c>
       <c r="E33" t="str">
         <v>admin1@sunrisevalley.com</v>
@@ -1584,7 +1584,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D34" t="str">
-        <v>Neeraj Kapoor</v>
+        <v>Chirag Das</v>
       </c>
       <c r="E34" t="str">
         <v>fm1@sunrisevalley.com</v>
@@ -1619,7 +1619,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D35" t="str">
-        <v>Farhan Choudhury</v>
+        <v>Chirag Menon</v>
       </c>
       <c r="E35" t="str">
         <v>guard1@sunrisevalley.com</v>
@@ -1654,7 +1654,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D36" t="str">
-        <v>Dev Mishra</v>
+        <v>Vishal Pillai</v>
       </c>
       <c r="E36" t="str">
         <v>guard2@sunrisevalley.com</v>
@@ -1689,7 +1689,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D37" t="str">
-        <v>Dev Singh</v>
+        <v>Gayatri Ghosh</v>
       </c>
       <c r="E37" t="str">
         <v>owner1@sunrisevalley.com</v>
@@ -1724,7 +1724,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D38" t="str">
-        <v>Sahil Agarwal</v>
+        <v>Varun Rao</v>
       </c>
       <c r="E38" t="str">
         <v>owner2@sunrisevalley.com</v>
@@ -1759,7 +1759,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D39" t="str">
-        <v>Vinay Agarwal</v>
+        <v>Neeraj Mishra</v>
       </c>
       <c r="E39" t="str">
         <v>owner3@sunrisevalley.com</v>
@@ -1794,7 +1794,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D40" t="str">
-        <v>Aarav Desai</v>
+        <v>Manav Banerjee</v>
       </c>
       <c r="E40" t="str">
         <v>owner4@sunrisevalley.com</v>
@@ -1829,7 +1829,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D41" t="str">
-        <v>Siddharth Shah</v>
+        <v>Yamini Iyer</v>
       </c>
       <c r="E41" t="str">
         <v>owner5@sunrisevalley.com</v>
@@ -1864,7 +1864,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D42" t="str">
-        <v>Kavya Singh</v>
+        <v>Manav Desai</v>
       </c>
       <c r="E42" t="str">
         <v>owner6@sunrisevalley.com</v>
@@ -1899,7 +1899,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D43" t="str">
-        <v>Nisha Bose</v>
+        <v>Chirag Iyer</v>
       </c>
       <c r="E43" t="str">
         <v>owner7@sunrisevalley.com</v>
@@ -1934,7 +1934,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D44" t="str">
-        <v>Tanvi Pillai</v>
+        <v>Seema Menon</v>
       </c>
       <c r="E44" t="str">
         <v>tenant1@sunrisevalley.com</v>
@@ -1969,7 +1969,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D45" t="str">
-        <v>Ananya Jain</v>
+        <v>Varun Iyer</v>
       </c>
       <c r="E45" t="str">
         <v>tenant2@sunrisevalley.com</v>
@@ -2004,7 +2004,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D46" t="str">
-        <v>Deepa Shah</v>
+        <v>Sangeeta Joshi</v>
       </c>
       <c r="E46" t="str">
         <v>tenant3@sunrisevalley.com</v>
@@ -2039,7 +2039,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D47" t="str">
-        <v>Pooja Kumar</v>
+        <v>Dev Pillai</v>
       </c>
       <c r="E47" t="str">
         <v>tenant4@sunrisevalley.com</v>
@@ -2074,7 +2074,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D48" t="str">
-        <v>Rohit Patel</v>
+        <v>Rajesh Choudhury</v>
       </c>
       <c r="E48" t="str">
         <v>tenant5@sunrisevalley.com</v>
@@ -2109,7 +2109,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D49" t="str">
-        <v>Lakshmi Sharma</v>
+        <v>Simran Mehta</v>
       </c>
       <c r="E49" t="str">
         <v>tenant6@sunrisevalley.com</v>
@@ -2144,7 +2144,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D50" t="str">
-        <v>Aarav Sinha</v>
+        <v>Yamini Menon</v>
       </c>
       <c r="E50" t="str">
         <v>tenant7@sunrisevalley.com</v>
@@ -2179,7 +2179,7 @@
         <v>Family Member</v>
       </c>
       <c r="D51" t="str">
-        <v>Zara Joshi</v>
+        <v>Sanjay Joshi</v>
       </c>
       <c r="E51" t="str">
         <v>family1@sunrisevalley.com</v>
@@ -2214,7 +2214,7 @@
         <v>Family Member</v>
       </c>
       <c r="D52" t="str">
-        <v>Jaya Kumar</v>
+        <v>Vishal Bhat</v>
       </c>
       <c r="E52" t="str">
         <v>family2@sunrisevalley.com</v>
@@ -2249,7 +2249,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D53" t="str">
-        <v>Rajesh Kapoor</v>
+        <v>Lakshmi Ghosh</v>
       </c>
       <c r="E53" t="str">
         <v>admin1@palmmeadows.com</v>
@@ -2284,7 +2284,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D54" t="str">
-        <v>Zara Iyer</v>
+        <v>Deepa Choudhury</v>
       </c>
       <c r="E54" t="str">
         <v>fm1@palmmeadows.com</v>
@@ -2319,7 +2319,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D55" t="str">
-        <v>Neeraj Menon</v>
+        <v>Pooja Das</v>
       </c>
       <c r="E55" t="str">
         <v>guard1@palmmeadows.com</v>
@@ -2354,7 +2354,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D56" t="str">
-        <v>Usha Rao</v>
+        <v>Harish Bhat</v>
       </c>
       <c r="E56" t="str">
         <v>owner1@palmmeadows.com</v>
@@ -2389,7 +2389,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D57" t="str">
-        <v>Sahil Chauhan</v>
+        <v>Sangeeta Pillai</v>
       </c>
       <c r="E57" t="str">
         <v>owner2@palmmeadows.com</v>
@@ -2424,7 +2424,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D58" t="str">
-        <v>Seema Banerjee</v>
+        <v>Varun Joshi</v>
       </c>
       <c r="E58" t="str">
         <v>owner3@palmmeadows.com</v>
@@ -2459,7 +2459,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D59" t="str">
-        <v>Tushar Sinha</v>
+        <v>Ananya Bhat</v>
       </c>
       <c r="E59" t="str">
         <v>owner4@palmmeadows.com</v>
@@ -2494,7 +2494,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D60" t="str">
-        <v>Shiv Shah</v>
+        <v>Pooja Tiwari</v>
       </c>
       <c r="E60" t="str">
         <v>owner5@palmmeadows.com</v>
@@ -2529,7 +2529,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D61" t="str">
-        <v>Siddharth Verma</v>
+        <v>Tanvi Nair</v>
       </c>
       <c r="E61" t="str">
         <v>tenant1@palmmeadows.com</v>
@@ -2564,7 +2564,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D62" t="str">
-        <v>Simran Tiwari</v>
+        <v>Sneha Bose</v>
       </c>
       <c r="E62" t="str">
         <v>tenant2@palmmeadows.com</v>
@@ -2599,7 +2599,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D63" t="str">
-        <v>Priya Das</v>
+        <v>Shiv Mehta</v>
       </c>
       <c r="E63" t="str">
         <v>tenant3@palmmeadows.com</v>
@@ -2634,7 +2634,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D64" t="str">
-        <v>Suresh Das</v>
+        <v>Siddharth Joshi</v>
       </c>
       <c r="E64" t="str">
         <v>tenant4@palmmeadows.com</v>
@@ -2669,7 +2669,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D65" t="str">
-        <v>Sangeeta Reddy</v>
+        <v>Akash Tiwari</v>
       </c>
       <c r="E65" t="str">
         <v>tenant5@palmmeadows.com</v>
@@ -2704,7 +2704,7 @@
         <v>Family Member</v>
       </c>
       <c r="D66" t="str">
-        <v>Vishal Kumar</v>
+        <v>Tushar Desai</v>
       </c>
       <c r="E66" t="str">
         <v>family1@palmmeadows.com</v>
@@ -2739,7 +2739,7 @@
         <v>Family Member</v>
       </c>
       <c r="D67" t="str">
-        <v>Arjun Rao</v>
+        <v>Arjun Mehta</v>
       </c>
       <c r="E67" t="str">
         <v>family2@palmmeadows.com</v>
@@ -2820,7 +2820,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Rohit Bose</v>
+        <v>Aarav Menon</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@greenfield.com</v>
@@ -2855,7 +2855,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D3" t="str">
-        <v>Harish Kumar</v>
+        <v>Rohit Gupta</v>
       </c>
       <c r="E3" t="str">
         <v>admin2@greenfield.com</v>
@@ -2890,7 +2890,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D4" t="str">
-        <v>Sanjay Kapoor</v>
+        <v>Rajesh Banerjee</v>
       </c>
       <c r="E4" t="str">
         <v>fm1@greenfield.com</v>
@@ -2925,7 +2925,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D5" t="str">
-        <v>Zara Sharma</v>
+        <v>Aarav Joshi</v>
       </c>
       <c r="E5" t="str">
         <v>fm2@greenfield.com</v>
@@ -2960,7 +2960,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D6" t="str">
-        <v>Vikram Mehta</v>
+        <v>Tanvi Bhat</v>
       </c>
       <c r="E6" t="str">
         <v>guard1@greenfield.com</v>
@@ -2995,7 +2995,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D7" t="str">
-        <v>Siddharth Gupta</v>
+        <v>Arjun Singh</v>
       </c>
       <c r="E7" t="str">
         <v>guard2@greenfield.com</v>
@@ -3030,7 +3030,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Ishaan Sinha</v>
+        <v>Sanjay Sharma</v>
       </c>
       <c r="E8" t="str">
         <v>owner1@greenfield.com</v>
@@ -3065,7 +3065,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Bhavna Shah</v>
+        <v>Akash Iyer</v>
       </c>
       <c r="E9" t="str">
         <v>owner2@greenfield.com</v>
@@ -3100,7 +3100,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Aditi Ghosh</v>
+        <v>Arjun Desai</v>
       </c>
       <c r="E10" t="str">
         <v>owner3@greenfield.com</v>
@@ -3135,7 +3135,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Rajesh Mehta</v>
+        <v>Yamini Bose</v>
       </c>
       <c r="E11" t="str">
         <v>owner4@greenfield.com</v>
@@ -3170,7 +3170,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Siddharth Iyer</v>
+        <v>Tanvi Iyer</v>
       </c>
       <c r="E12" t="str">
         <v>owner5@greenfield.com</v>
@@ -3205,7 +3205,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D13" t="str">
-        <v>Rahul Patel</v>
+        <v>Rekha Mishra</v>
       </c>
       <c r="E13" t="str">
         <v>owner6@greenfield.com</v>
@@ -3240,7 +3240,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D14" t="str">
-        <v>Priya Verma</v>
+        <v>Ananya Iyer</v>
       </c>
       <c r="E14" t="str">
         <v>owner7@greenfield.com</v>
@@ -3275,7 +3275,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D15" t="str">
-        <v>Tanvi Shah</v>
+        <v>Rahul Verma</v>
       </c>
       <c r="E15" t="str">
         <v>owner8@greenfield.com</v>
@@ -3310,7 +3310,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D16" t="str">
-        <v>Jaya Mehta</v>
+        <v>Sanjay Mehta</v>
       </c>
       <c r="E16" t="str">
         <v>owner9@greenfield.com</v>
@@ -3345,7 +3345,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D17" t="str">
-        <v>Sahil Kumar</v>
+        <v>Sahil Rao</v>
       </c>
       <c r="E17" t="str">
         <v>owner10@greenfield.com</v>
@@ -3380,7 +3380,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D18" t="str">
-        <v>Siddharth Mehta</v>
+        <v>Om Banerjee</v>
       </c>
       <c r="E18" t="str">
         <v>tenant1@greenfield.com</v>
@@ -3415,7 +3415,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Harish Banerjee</v>
+        <v>Aditi Agarwal</v>
       </c>
       <c r="E19" t="str">
         <v>tenant2@greenfield.com</v>
@@ -3450,7 +3450,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D20" t="str">
-        <v>Chirag Rao</v>
+        <v>Rajesh Pillai</v>
       </c>
       <c r="E20" t="str">
         <v>tenant3@greenfield.com</v>
@@ -3485,7 +3485,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D21" t="str">
-        <v>Yamini Gupta</v>
+        <v>Meera Patel</v>
       </c>
       <c r="E21" t="str">
         <v>tenant4@greenfield.com</v>
@@ -3520,7 +3520,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D22" t="str">
-        <v>Rajesh Banerjee</v>
+        <v>Vikram Singh</v>
       </c>
       <c r="E22" t="str">
         <v>tenant5@greenfield.com</v>
@@ -3555,7 +3555,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D23" t="str">
-        <v>Kavya Patel</v>
+        <v>Shiv Reddy</v>
       </c>
       <c r="E23" t="str">
         <v>tenant6@greenfield.com</v>
@@ -3590,7 +3590,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D24" t="str">
-        <v>Ananya Banerjee</v>
+        <v>Arjun Verma</v>
       </c>
       <c r="E24" t="str">
         <v>tenant7@greenfield.com</v>
@@ -3625,7 +3625,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D25" t="str">
-        <v>Vinay Banerjee</v>
+        <v>Priya Ghosh</v>
       </c>
       <c r="E25" t="str">
         <v>tenant8@greenfield.com</v>
@@ -3660,7 +3660,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D26" t="str">
-        <v>Divya Singh</v>
+        <v>Meera Mehta</v>
       </c>
       <c r="E26" t="str">
         <v>tenant9@greenfield.com</v>
@@ -3695,7 +3695,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D27" t="str">
-        <v>Kavya Bose</v>
+        <v>Jaya Kumar</v>
       </c>
       <c r="E27" t="str">
         <v>tenant10@greenfield.com</v>
@@ -3730,7 +3730,7 @@
         <v>Family Member</v>
       </c>
       <c r="D28" t="str">
-        <v>Farhan Pandey</v>
+        <v>Divya Bose</v>
       </c>
       <c r="E28" t="str">
         <v>family1@greenfield.com</v>
@@ -3765,7 +3765,7 @@
         <v>Family Member</v>
       </c>
       <c r="D29" t="str">
-        <v>Varun Ghosh</v>
+        <v>Ishaan Sharma</v>
       </c>
       <c r="E29" t="str">
         <v>family2@greenfield.com</v>
@@ -3800,7 +3800,7 @@
         <v>Family Member</v>
       </c>
       <c r="D30" t="str">
-        <v>Nisha Rao</v>
+        <v>Zara Verma</v>
       </c>
       <c r="E30" t="str">
         <v>family3@greenfield.com</v>
@@ -3835,7 +3835,7 @@
         <v>Family Member</v>
       </c>
       <c r="D31" t="str">
-        <v>Rajesh Nair</v>
+        <v>Chirag Bhat</v>
       </c>
       <c r="E31" t="str">
         <v>family4@greenfield.com</v>
@@ -3916,7 +3916,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Varun Pandey</v>
+        <v>Karan Pillai</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@sunrisevalley.com</v>
@@ -3951,7 +3951,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D3" t="str">
-        <v>Neeraj Kapoor</v>
+        <v>Chirag Das</v>
       </c>
       <c r="E3" t="str">
         <v>fm1@sunrisevalley.com</v>
@@ -3986,7 +3986,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D4" t="str">
-        <v>Farhan Choudhury</v>
+        <v>Chirag Menon</v>
       </c>
       <c r="E4" t="str">
         <v>guard1@sunrisevalley.com</v>
@@ -4021,7 +4021,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D5" t="str">
-        <v>Dev Mishra</v>
+        <v>Vishal Pillai</v>
       </c>
       <c r="E5" t="str">
         <v>guard2@sunrisevalley.com</v>
@@ -4056,7 +4056,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D6" t="str">
-        <v>Dev Singh</v>
+        <v>Gayatri Ghosh</v>
       </c>
       <c r="E6" t="str">
         <v>owner1@sunrisevalley.com</v>
@@ -4091,7 +4091,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D7" t="str">
-        <v>Sahil Agarwal</v>
+        <v>Varun Rao</v>
       </c>
       <c r="E7" t="str">
         <v>owner2@sunrisevalley.com</v>
@@ -4126,7 +4126,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Vinay Agarwal</v>
+        <v>Neeraj Mishra</v>
       </c>
       <c r="E8" t="str">
         <v>owner3@sunrisevalley.com</v>
@@ -4161,7 +4161,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Aarav Desai</v>
+        <v>Manav Banerjee</v>
       </c>
       <c r="E9" t="str">
         <v>owner4@sunrisevalley.com</v>
@@ -4196,7 +4196,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Siddharth Shah</v>
+        <v>Yamini Iyer</v>
       </c>
       <c r="E10" t="str">
         <v>owner5@sunrisevalley.com</v>
@@ -4231,7 +4231,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Kavya Singh</v>
+        <v>Manav Desai</v>
       </c>
       <c r="E11" t="str">
         <v>owner6@sunrisevalley.com</v>
@@ -4266,7 +4266,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Nisha Bose</v>
+        <v>Chirag Iyer</v>
       </c>
       <c r="E12" t="str">
         <v>owner7@sunrisevalley.com</v>
@@ -4301,7 +4301,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D13" t="str">
-        <v>Tanvi Pillai</v>
+        <v>Seema Menon</v>
       </c>
       <c r="E13" t="str">
         <v>tenant1@sunrisevalley.com</v>
@@ -4336,7 +4336,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D14" t="str">
-        <v>Ananya Jain</v>
+        <v>Varun Iyer</v>
       </c>
       <c r="E14" t="str">
         <v>tenant2@sunrisevalley.com</v>
@@ -4371,7 +4371,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D15" t="str">
-        <v>Deepa Shah</v>
+        <v>Sangeeta Joshi</v>
       </c>
       <c r="E15" t="str">
         <v>tenant3@sunrisevalley.com</v>
@@ -4406,7 +4406,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D16" t="str">
-        <v>Pooja Kumar</v>
+        <v>Dev Pillai</v>
       </c>
       <c r="E16" t="str">
         <v>tenant4@sunrisevalley.com</v>
@@ -4441,7 +4441,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D17" t="str">
-        <v>Rohit Patel</v>
+        <v>Rajesh Choudhury</v>
       </c>
       <c r="E17" t="str">
         <v>tenant5@sunrisevalley.com</v>
@@ -4476,7 +4476,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D18" t="str">
-        <v>Lakshmi Sharma</v>
+        <v>Simran Mehta</v>
       </c>
       <c r="E18" t="str">
         <v>tenant6@sunrisevalley.com</v>
@@ -4511,7 +4511,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Aarav Sinha</v>
+        <v>Yamini Menon</v>
       </c>
       <c r="E19" t="str">
         <v>tenant7@sunrisevalley.com</v>
@@ -4546,7 +4546,7 @@
         <v>Family Member</v>
       </c>
       <c r="D20" t="str">
-        <v>Zara Joshi</v>
+        <v>Sanjay Joshi</v>
       </c>
       <c r="E20" t="str">
         <v>family1@sunrisevalley.com</v>
@@ -4581,7 +4581,7 @@
         <v>Family Member</v>
       </c>
       <c r="D21" t="str">
-        <v>Jaya Kumar</v>
+        <v>Vishal Bhat</v>
       </c>
       <c r="E21" t="str">
         <v>family2@sunrisevalley.com</v>
@@ -4662,7 +4662,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Rajesh Kapoor</v>
+        <v>Lakshmi Ghosh</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@palmmeadows.com</v>
@@ -4697,7 +4697,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D3" t="str">
-        <v>Zara Iyer</v>
+        <v>Deepa Choudhury</v>
       </c>
       <c r="E3" t="str">
         <v>fm1@palmmeadows.com</v>
@@ -4732,7 +4732,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D4" t="str">
-        <v>Neeraj Menon</v>
+        <v>Pooja Das</v>
       </c>
       <c r="E4" t="str">
         <v>guard1@palmmeadows.com</v>
@@ -4767,7 +4767,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D5" t="str">
-        <v>Usha Rao</v>
+        <v>Harish Bhat</v>
       </c>
       <c r="E5" t="str">
         <v>owner1@palmmeadows.com</v>
@@ -4802,7 +4802,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D6" t="str">
-        <v>Sahil Chauhan</v>
+        <v>Sangeeta Pillai</v>
       </c>
       <c r="E6" t="str">
         <v>owner2@palmmeadows.com</v>
@@ -4837,7 +4837,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D7" t="str">
-        <v>Seema Banerjee</v>
+        <v>Varun Joshi</v>
       </c>
       <c r="E7" t="str">
         <v>owner3@palmmeadows.com</v>
@@ -4872,7 +4872,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Tushar Sinha</v>
+        <v>Ananya Bhat</v>
       </c>
       <c r="E8" t="str">
         <v>owner4@palmmeadows.com</v>
@@ -4907,7 +4907,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Shiv Shah</v>
+        <v>Pooja Tiwari</v>
       </c>
       <c r="E9" t="str">
         <v>owner5@palmmeadows.com</v>
@@ -4942,7 +4942,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D10" t="str">
-        <v>Siddharth Verma</v>
+        <v>Tanvi Nair</v>
       </c>
       <c r="E10" t="str">
         <v>tenant1@palmmeadows.com</v>
@@ -4977,7 +4977,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D11" t="str">
-        <v>Simran Tiwari</v>
+        <v>Sneha Bose</v>
       </c>
       <c r="E11" t="str">
         <v>tenant2@palmmeadows.com</v>
@@ -5012,7 +5012,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D12" t="str">
-        <v>Priya Das</v>
+        <v>Shiv Mehta</v>
       </c>
       <c r="E12" t="str">
         <v>tenant3@palmmeadows.com</v>
@@ -5047,7 +5047,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D13" t="str">
-        <v>Suresh Das</v>
+        <v>Siddharth Joshi</v>
       </c>
       <c r="E13" t="str">
         <v>tenant4@palmmeadows.com</v>
@@ -5082,7 +5082,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D14" t="str">
-        <v>Sangeeta Reddy</v>
+        <v>Akash Tiwari</v>
       </c>
       <c r="E14" t="str">
         <v>tenant5@palmmeadows.com</v>
@@ -5117,7 +5117,7 @@
         <v>Family Member</v>
       </c>
       <c r="D15" t="str">
-        <v>Vishal Kumar</v>
+        <v>Tushar Desai</v>
       </c>
       <c r="E15" t="str">
         <v>family1@palmmeadows.com</v>
@@ -5152,7 +5152,7 @@
         <v>Family Member</v>
       </c>
       <c r="D16" t="str">
-        <v>Arjun Rao</v>
+        <v>Arjun Mehta</v>
       </c>
       <c r="E16" t="str">
         <v>family2@palmmeadows.com</v>
@@ -5322,7 +5322,7 @@
         <v>Platform Multi-Community Switch</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login with admin@enterprise.com / SuperAdminPwd@123.
+        <v xml:space="preserve">1. Login with admin@managemygate.com / password123.
 2. Open workspace dropdown in header.
 3. Verify all 3 communities (Greenfield Heights, Sunrise Valley, Palm Meadows) are listed.
 4. Switch workspace and verify context changes.</v>
@@ -5517,7 +5517,7 @@
         <v>Super Admin Account</v>
       </c>
       <c r="B7" t="str">
-        <v>admin@enterprise.com (Password: SuperAdminPwd@123)</v>
+        <v>admin@managemygate.com (Password: password123)</v>
       </c>
     </row>
     <row r="8">
@@ -5541,7 +5541,7 @@
         <v>Seed Execution Timestamp</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-07-31T10:38:45.636Z</v>
+        <v>2026-08-20T09:13:54.920Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(mobile): update UI branding, component catalog, and screen design system
</commit_message>
<xml_diff>
--- a/Community_Testing_Credentials.xlsx
+++ b/Community_Testing_Credentials.xlsx
@@ -499,7 +499,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D3" t="str">
-        <v>Aarav Menon</v>
+        <v>Sapna Singh</v>
       </c>
       <c r="E3" t="str">
         <v>admin1@greenfield.com</v>
@@ -534,7 +534,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D4" t="str">
-        <v>Rohit Gupta</v>
+        <v>Shreya Bhat</v>
       </c>
       <c r="E4" t="str">
         <v>admin2@greenfield.com</v>
@@ -569,7 +569,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D5" t="str">
-        <v>Rajesh Banerjee</v>
+        <v>Suresh Verma</v>
       </c>
       <c r="E5" t="str">
         <v>fm1@greenfield.com</v>
@@ -604,7 +604,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D6" t="str">
-        <v>Aarav Joshi</v>
+        <v>Dev Tiwari</v>
       </c>
       <c r="E6" t="str">
         <v>fm2@greenfield.com</v>
@@ -639,7 +639,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D7" t="str">
-        <v>Tanvi Bhat</v>
+        <v>Meera Sinha</v>
       </c>
       <c r="E7" t="str">
         <v>guard1@greenfield.com</v>
@@ -674,7 +674,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D8" t="str">
-        <v>Arjun Singh</v>
+        <v>Arjun Jain</v>
       </c>
       <c r="E8" t="str">
         <v>guard2@greenfield.com</v>
@@ -709,7 +709,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Sanjay Sharma</v>
+        <v>Karan Rao</v>
       </c>
       <c r="E9" t="str">
         <v>owner1@greenfield.com</v>
@@ -744,7 +744,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Akash Iyer</v>
+        <v>Akash Joshi</v>
       </c>
       <c r="E10" t="str">
         <v>owner2@greenfield.com</v>
@@ -779,7 +779,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Arjun Desai</v>
+        <v>Siddharth Sharma</v>
       </c>
       <c r="E11" t="str">
         <v>owner3@greenfield.com</v>
@@ -814,7 +814,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Yamini Bose</v>
+        <v>Ananya Pillai</v>
       </c>
       <c r="E12" t="str">
         <v>owner4@greenfield.com</v>
@@ -849,7 +849,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D13" t="str">
-        <v>Tanvi Iyer</v>
+        <v>Vinay Sharma</v>
       </c>
       <c r="E13" t="str">
         <v>owner5@greenfield.com</v>
@@ -884,7 +884,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D14" t="str">
-        <v>Rekha Mishra</v>
+        <v>Pranav Kapoor</v>
       </c>
       <c r="E14" t="str">
         <v>owner6@greenfield.com</v>
@@ -919,7 +919,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D15" t="str">
-        <v>Ananya Iyer</v>
+        <v>Meera Iyer</v>
       </c>
       <c r="E15" t="str">
         <v>owner7@greenfield.com</v>
@@ -954,7 +954,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D16" t="str">
-        <v>Rahul Verma</v>
+        <v>Seema Menon</v>
       </c>
       <c r="E16" t="str">
         <v>owner8@greenfield.com</v>
@@ -989,7 +989,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D17" t="str">
-        <v>Sanjay Mehta</v>
+        <v>Divya Pandey</v>
       </c>
       <c r="E17" t="str">
         <v>owner9@greenfield.com</v>
@@ -1024,7 +1024,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D18" t="str">
-        <v>Sahil Rao</v>
+        <v>Vinay Das</v>
       </c>
       <c r="E18" t="str">
         <v>owner10@greenfield.com</v>
@@ -1059,7 +1059,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Om Banerjee</v>
+        <v>Priya Reddy</v>
       </c>
       <c r="E19" t="str">
         <v>tenant1@greenfield.com</v>
@@ -1094,7 +1094,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D20" t="str">
-        <v>Aditi Agarwal</v>
+        <v>Priya Mishra</v>
       </c>
       <c r="E20" t="str">
         <v>tenant2@greenfield.com</v>
@@ -1129,7 +1129,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D21" t="str">
-        <v>Rajesh Pillai</v>
+        <v>Ananya Pillai</v>
       </c>
       <c r="E21" t="str">
         <v>tenant3@greenfield.com</v>
@@ -1164,7 +1164,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D22" t="str">
-        <v>Meera Patel</v>
+        <v>Shreya Chauhan</v>
       </c>
       <c r="E22" t="str">
         <v>tenant4@greenfield.com</v>
@@ -1199,7 +1199,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D23" t="str">
-        <v>Vikram Singh</v>
+        <v>Rekha Pandey</v>
       </c>
       <c r="E23" t="str">
         <v>tenant5@greenfield.com</v>
@@ -1234,7 +1234,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D24" t="str">
-        <v>Shiv Reddy</v>
+        <v>Priya Mehta</v>
       </c>
       <c r="E24" t="str">
         <v>tenant6@greenfield.com</v>
@@ -1269,7 +1269,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D25" t="str">
-        <v>Arjun Verma</v>
+        <v>Manav Jain</v>
       </c>
       <c r="E25" t="str">
         <v>tenant7@greenfield.com</v>
@@ -1304,7 +1304,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D26" t="str">
-        <v>Priya Ghosh</v>
+        <v>Sangeeta Pillai</v>
       </c>
       <c r="E26" t="str">
         <v>tenant8@greenfield.com</v>
@@ -1339,7 +1339,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D27" t="str">
-        <v>Meera Mehta</v>
+        <v>Nisha Pandey</v>
       </c>
       <c r="E27" t="str">
         <v>tenant9@greenfield.com</v>
@@ -1374,7 +1374,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D28" t="str">
-        <v>Jaya Kumar</v>
+        <v>Karan Bhat</v>
       </c>
       <c r="E28" t="str">
         <v>tenant10@greenfield.com</v>
@@ -1409,7 +1409,7 @@
         <v>Family Member</v>
       </c>
       <c r="D29" t="str">
-        <v>Divya Bose</v>
+        <v>Siddharth Mehta</v>
       </c>
       <c r="E29" t="str">
         <v>family1@greenfield.com</v>
@@ -1444,7 +1444,7 @@
         <v>Family Member</v>
       </c>
       <c r="D30" t="str">
-        <v>Ishaan Sharma</v>
+        <v>Tanvi Ghosh</v>
       </c>
       <c r="E30" t="str">
         <v>family2@greenfield.com</v>
@@ -1479,7 +1479,7 @@
         <v>Family Member</v>
       </c>
       <c r="D31" t="str">
-        <v>Zara Verma</v>
+        <v>Pranav Bose</v>
       </c>
       <c r="E31" t="str">
         <v>family3@greenfield.com</v>
@@ -1514,7 +1514,7 @@
         <v>Family Member</v>
       </c>
       <c r="D32" t="str">
-        <v>Chirag Bhat</v>
+        <v>Ananya Verma</v>
       </c>
       <c r="E32" t="str">
         <v>family4@greenfield.com</v>
@@ -1549,7 +1549,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D33" t="str">
-        <v>Karan Pillai</v>
+        <v>Aditi Bose</v>
       </c>
       <c r="E33" t="str">
         <v>admin1@sunrisevalley.com</v>
@@ -1584,7 +1584,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D34" t="str">
-        <v>Chirag Das</v>
+        <v>Manav Pandey</v>
       </c>
       <c r="E34" t="str">
         <v>fm1@sunrisevalley.com</v>
@@ -1619,7 +1619,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D35" t="str">
-        <v>Chirag Menon</v>
+        <v>Sangeeta Pandey</v>
       </c>
       <c r="E35" t="str">
         <v>guard1@sunrisevalley.com</v>
@@ -1654,7 +1654,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D36" t="str">
-        <v>Vishal Pillai</v>
+        <v>Yamini Agarwal</v>
       </c>
       <c r="E36" t="str">
         <v>guard2@sunrisevalley.com</v>
@@ -1689,7 +1689,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D37" t="str">
-        <v>Gayatri Ghosh</v>
+        <v>Dev Nair</v>
       </c>
       <c r="E37" t="str">
         <v>owner1@sunrisevalley.com</v>
@@ -1724,7 +1724,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D38" t="str">
-        <v>Varun Rao</v>
+        <v>Harish Rao</v>
       </c>
       <c r="E38" t="str">
         <v>owner2@sunrisevalley.com</v>
@@ -1759,7 +1759,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D39" t="str">
-        <v>Neeraj Mishra</v>
+        <v>Ananya Desai</v>
       </c>
       <c r="E39" t="str">
         <v>owner3@sunrisevalley.com</v>
@@ -1794,7 +1794,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D40" t="str">
-        <v>Manav Banerjee</v>
+        <v>Zara Mehta</v>
       </c>
       <c r="E40" t="str">
         <v>owner4@sunrisevalley.com</v>
@@ -1829,7 +1829,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D41" t="str">
-        <v>Yamini Iyer</v>
+        <v>Tanvi Joshi</v>
       </c>
       <c r="E41" t="str">
         <v>owner5@sunrisevalley.com</v>
@@ -1864,7 +1864,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D42" t="str">
-        <v>Manav Desai</v>
+        <v>Gayatri Kapoor</v>
       </c>
       <c r="E42" t="str">
         <v>owner6@sunrisevalley.com</v>
@@ -1899,7 +1899,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D43" t="str">
-        <v>Chirag Iyer</v>
+        <v>Kavya Bhat</v>
       </c>
       <c r="E43" t="str">
         <v>owner7@sunrisevalley.com</v>
@@ -1934,7 +1934,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D44" t="str">
-        <v>Seema Menon</v>
+        <v>Usha Chauhan</v>
       </c>
       <c r="E44" t="str">
         <v>tenant1@sunrisevalley.com</v>
@@ -1969,7 +1969,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D45" t="str">
-        <v>Varun Iyer</v>
+        <v>Vinay Chauhan</v>
       </c>
       <c r="E45" t="str">
         <v>tenant2@sunrisevalley.com</v>
@@ -2004,7 +2004,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D46" t="str">
-        <v>Sangeeta Joshi</v>
+        <v>Priya Desai</v>
       </c>
       <c r="E46" t="str">
         <v>tenant3@sunrisevalley.com</v>
@@ -2039,7 +2039,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D47" t="str">
-        <v>Dev Pillai</v>
+        <v>Vikram Nair</v>
       </c>
       <c r="E47" t="str">
         <v>tenant4@sunrisevalley.com</v>
@@ -2074,7 +2074,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D48" t="str">
-        <v>Rajesh Choudhury</v>
+        <v>Usha Iyer</v>
       </c>
       <c r="E48" t="str">
         <v>tenant5@sunrisevalley.com</v>
@@ -2109,7 +2109,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D49" t="str">
-        <v>Simran Mehta</v>
+        <v>Shreya Reddy</v>
       </c>
       <c r="E49" t="str">
         <v>tenant6@sunrisevalley.com</v>
@@ -2144,7 +2144,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D50" t="str">
-        <v>Yamini Menon</v>
+        <v>Bhavna Agarwal</v>
       </c>
       <c r="E50" t="str">
         <v>tenant7@sunrisevalley.com</v>
@@ -2179,7 +2179,7 @@
         <v>Family Member</v>
       </c>
       <c r="D51" t="str">
-        <v>Sanjay Joshi</v>
+        <v>Rohit Chauhan</v>
       </c>
       <c r="E51" t="str">
         <v>family1@sunrisevalley.com</v>
@@ -2214,7 +2214,7 @@
         <v>Family Member</v>
       </c>
       <c r="D52" t="str">
-        <v>Vishal Bhat</v>
+        <v>Bhavna Patel</v>
       </c>
       <c r="E52" t="str">
         <v>family2@sunrisevalley.com</v>
@@ -2249,7 +2249,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D53" t="str">
-        <v>Lakshmi Ghosh</v>
+        <v>Aditi Rao</v>
       </c>
       <c r="E53" t="str">
         <v>admin1@palmmeadows.com</v>
@@ -2284,7 +2284,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D54" t="str">
-        <v>Deepa Choudhury</v>
+        <v>Vinay Desai</v>
       </c>
       <c r="E54" t="str">
         <v>fm1@palmmeadows.com</v>
@@ -2319,7 +2319,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D55" t="str">
-        <v>Pooja Das</v>
+        <v>Rajesh Bose</v>
       </c>
       <c r="E55" t="str">
         <v>guard1@palmmeadows.com</v>
@@ -2354,7 +2354,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D56" t="str">
-        <v>Harish Bhat</v>
+        <v>Meera Nair</v>
       </c>
       <c r="E56" t="str">
         <v>owner1@palmmeadows.com</v>
@@ -2389,7 +2389,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D57" t="str">
-        <v>Sangeeta Pillai</v>
+        <v>Ananya Patel</v>
       </c>
       <c r="E57" t="str">
         <v>owner2@palmmeadows.com</v>
@@ -2424,7 +2424,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D58" t="str">
-        <v>Varun Joshi</v>
+        <v>Yamini Bose</v>
       </c>
       <c r="E58" t="str">
         <v>owner3@palmmeadows.com</v>
@@ -2459,7 +2459,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D59" t="str">
-        <v>Ananya Bhat</v>
+        <v>Farhan Reddy</v>
       </c>
       <c r="E59" t="str">
         <v>owner4@palmmeadows.com</v>
@@ -2494,7 +2494,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D60" t="str">
-        <v>Pooja Tiwari</v>
+        <v>Farhan Tiwari</v>
       </c>
       <c r="E60" t="str">
         <v>owner5@palmmeadows.com</v>
@@ -2529,7 +2529,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D61" t="str">
-        <v>Tanvi Nair</v>
+        <v>Vishal Jain</v>
       </c>
       <c r="E61" t="str">
         <v>tenant1@palmmeadows.com</v>
@@ -2564,7 +2564,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D62" t="str">
-        <v>Sneha Bose</v>
+        <v>Karan Iyer</v>
       </c>
       <c r="E62" t="str">
         <v>tenant2@palmmeadows.com</v>
@@ -2599,7 +2599,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D63" t="str">
-        <v>Shiv Mehta</v>
+        <v>Siddharth Verma</v>
       </c>
       <c r="E63" t="str">
         <v>tenant3@palmmeadows.com</v>
@@ -2634,7 +2634,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D64" t="str">
-        <v>Siddharth Joshi</v>
+        <v>Bhavna Bhat</v>
       </c>
       <c r="E64" t="str">
         <v>tenant4@palmmeadows.com</v>
@@ -2669,7 +2669,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D65" t="str">
-        <v>Akash Tiwari</v>
+        <v>Shiv Nair</v>
       </c>
       <c r="E65" t="str">
         <v>tenant5@palmmeadows.com</v>
@@ -2704,7 +2704,7 @@
         <v>Family Member</v>
       </c>
       <c r="D66" t="str">
-        <v>Tushar Desai</v>
+        <v>Arjun Patel</v>
       </c>
       <c r="E66" t="str">
         <v>family1@palmmeadows.com</v>
@@ -2739,7 +2739,7 @@
         <v>Family Member</v>
       </c>
       <c r="D67" t="str">
-        <v>Arjun Mehta</v>
+        <v>Pranav Kumar</v>
       </c>
       <c r="E67" t="str">
         <v>family2@palmmeadows.com</v>
@@ -2820,7 +2820,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Aarav Menon</v>
+        <v>Sapna Singh</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@greenfield.com</v>
@@ -2855,7 +2855,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D3" t="str">
-        <v>Rohit Gupta</v>
+        <v>Shreya Bhat</v>
       </c>
       <c r="E3" t="str">
         <v>admin2@greenfield.com</v>
@@ -2890,7 +2890,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D4" t="str">
-        <v>Rajesh Banerjee</v>
+        <v>Suresh Verma</v>
       </c>
       <c r="E4" t="str">
         <v>fm1@greenfield.com</v>
@@ -2925,7 +2925,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D5" t="str">
-        <v>Aarav Joshi</v>
+        <v>Dev Tiwari</v>
       </c>
       <c r="E5" t="str">
         <v>fm2@greenfield.com</v>
@@ -2960,7 +2960,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D6" t="str">
-        <v>Tanvi Bhat</v>
+        <v>Meera Sinha</v>
       </c>
       <c r="E6" t="str">
         <v>guard1@greenfield.com</v>
@@ -2995,7 +2995,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D7" t="str">
-        <v>Arjun Singh</v>
+        <v>Arjun Jain</v>
       </c>
       <c r="E7" t="str">
         <v>guard2@greenfield.com</v>
@@ -3030,7 +3030,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Sanjay Sharma</v>
+        <v>Karan Rao</v>
       </c>
       <c r="E8" t="str">
         <v>owner1@greenfield.com</v>
@@ -3065,7 +3065,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Akash Iyer</v>
+        <v>Akash Joshi</v>
       </c>
       <c r="E9" t="str">
         <v>owner2@greenfield.com</v>
@@ -3100,7 +3100,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Arjun Desai</v>
+        <v>Siddharth Sharma</v>
       </c>
       <c r="E10" t="str">
         <v>owner3@greenfield.com</v>
@@ -3135,7 +3135,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Yamini Bose</v>
+        <v>Ananya Pillai</v>
       </c>
       <c r="E11" t="str">
         <v>owner4@greenfield.com</v>
@@ -3170,7 +3170,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Tanvi Iyer</v>
+        <v>Vinay Sharma</v>
       </c>
       <c r="E12" t="str">
         <v>owner5@greenfield.com</v>
@@ -3205,7 +3205,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D13" t="str">
-        <v>Rekha Mishra</v>
+        <v>Pranav Kapoor</v>
       </c>
       <c r="E13" t="str">
         <v>owner6@greenfield.com</v>
@@ -3240,7 +3240,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D14" t="str">
-        <v>Ananya Iyer</v>
+        <v>Meera Iyer</v>
       </c>
       <c r="E14" t="str">
         <v>owner7@greenfield.com</v>
@@ -3275,7 +3275,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D15" t="str">
-        <v>Rahul Verma</v>
+        <v>Seema Menon</v>
       </c>
       <c r="E15" t="str">
         <v>owner8@greenfield.com</v>
@@ -3310,7 +3310,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D16" t="str">
-        <v>Sanjay Mehta</v>
+        <v>Divya Pandey</v>
       </c>
       <c r="E16" t="str">
         <v>owner9@greenfield.com</v>
@@ -3345,7 +3345,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D17" t="str">
-        <v>Sahil Rao</v>
+        <v>Vinay Das</v>
       </c>
       <c r="E17" t="str">
         <v>owner10@greenfield.com</v>
@@ -3380,7 +3380,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D18" t="str">
-        <v>Om Banerjee</v>
+        <v>Priya Reddy</v>
       </c>
       <c r="E18" t="str">
         <v>tenant1@greenfield.com</v>
@@ -3415,7 +3415,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Aditi Agarwal</v>
+        <v>Priya Mishra</v>
       </c>
       <c r="E19" t="str">
         <v>tenant2@greenfield.com</v>
@@ -3450,7 +3450,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D20" t="str">
-        <v>Rajesh Pillai</v>
+        <v>Ananya Pillai</v>
       </c>
       <c r="E20" t="str">
         <v>tenant3@greenfield.com</v>
@@ -3485,7 +3485,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D21" t="str">
-        <v>Meera Patel</v>
+        <v>Shreya Chauhan</v>
       </c>
       <c r="E21" t="str">
         <v>tenant4@greenfield.com</v>
@@ -3520,7 +3520,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D22" t="str">
-        <v>Vikram Singh</v>
+        <v>Rekha Pandey</v>
       </c>
       <c r="E22" t="str">
         <v>tenant5@greenfield.com</v>
@@ -3555,7 +3555,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D23" t="str">
-        <v>Shiv Reddy</v>
+        <v>Priya Mehta</v>
       </c>
       <c r="E23" t="str">
         <v>tenant6@greenfield.com</v>
@@ -3590,7 +3590,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D24" t="str">
-        <v>Arjun Verma</v>
+        <v>Manav Jain</v>
       </c>
       <c r="E24" t="str">
         <v>tenant7@greenfield.com</v>
@@ -3625,7 +3625,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D25" t="str">
-        <v>Priya Ghosh</v>
+        <v>Sangeeta Pillai</v>
       </c>
       <c r="E25" t="str">
         <v>tenant8@greenfield.com</v>
@@ -3660,7 +3660,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D26" t="str">
-        <v>Meera Mehta</v>
+        <v>Nisha Pandey</v>
       </c>
       <c r="E26" t="str">
         <v>tenant9@greenfield.com</v>
@@ -3695,7 +3695,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D27" t="str">
-        <v>Jaya Kumar</v>
+        <v>Karan Bhat</v>
       </c>
       <c r="E27" t="str">
         <v>tenant10@greenfield.com</v>
@@ -3730,7 +3730,7 @@
         <v>Family Member</v>
       </c>
       <c r="D28" t="str">
-        <v>Divya Bose</v>
+        <v>Siddharth Mehta</v>
       </c>
       <c r="E28" t="str">
         <v>family1@greenfield.com</v>
@@ -3765,7 +3765,7 @@
         <v>Family Member</v>
       </c>
       <c r="D29" t="str">
-        <v>Ishaan Sharma</v>
+        <v>Tanvi Ghosh</v>
       </c>
       <c r="E29" t="str">
         <v>family2@greenfield.com</v>
@@ -3800,7 +3800,7 @@
         <v>Family Member</v>
       </c>
       <c r="D30" t="str">
-        <v>Zara Verma</v>
+        <v>Pranav Bose</v>
       </c>
       <c r="E30" t="str">
         <v>family3@greenfield.com</v>
@@ -3835,7 +3835,7 @@
         <v>Family Member</v>
       </c>
       <c r="D31" t="str">
-        <v>Chirag Bhat</v>
+        <v>Ananya Verma</v>
       </c>
       <c r="E31" t="str">
         <v>family4@greenfield.com</v>
@@ -3916,7 +3916,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Karan Pillai</v>
+        <v>Aditi Bose</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@sunrisevalley.com</v>
@@ -3951,7 +3951,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D3" t="str">
-        <v>Chirag Das</v>
+        <v>Manav Pandey</v>
       </c>
       <c r="E3" t="str">
         <v>fm1@sunrisevalley.com</v>
@@ -3986,7 +3986,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D4" t="str">
-        <v>Chirag Menon</v>
+        <v>Sangeeta Pandey</v>
       </c>
       <c r="E4" t="str">
         <v>guard1@sunrisevalley.com</v>
@@ -4021,7 +4021,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D5" t="str">
-        <v>Vishal Pillai</v>
+        <v>Yamini Agarwal</v>
       </c>
       <c r="E5" t="str">
         <v>guard2@sunrisevalley.com</v>
@@ -4056,7 +4056,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D6" t="str">
-        <v>Gayatri Ghosh</v>
+        <v>Dev Nair</v>
       </c>
       <c r="E6" t="str">
         <v>owner1@sunrisevalley.com</v>
@@ -4091,7 +4091,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D7" t="str">
-        <v>Varun Rao</v>
+        <v>Harish Rao</v>
       </c>
       <c r="E7" t="str">
         <v>owner2@sunrisevalley.com</v>
@@ -4126,7 +4126,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Neeraj Mishra</v>
+        <v>Ananya Desai</v>
       </c>
       <c r="E8" t="str">
         <v>owner3@sunrisevalley.com</v>
@@ -4161,7 +4161,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Manav Banerjee</v>
+        <v>Zara Mehta</v>
       </c>
       <c r="E9" t="str">
         <v>owner4@sunrisevalley.com</v>
@@ -4196,7 +4196,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Yamini Iyer</v>
+        <v>Tanvi Joshi</v>
       </c>
       <c r="E10" t="str">
         <v>owner5@sunrisevalley.com</v>
@@ -4231,7 +4231,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Manav Desai</v>
+        <v>Gayatri Kapoor</v>
       </c>
       <c r="E11" t="str">
         <v>owner6@sunrisevalley.com</v>
@@ -4266,7 +4266,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Chirag Iyer</v>
+        <v>Kavya Bhat</v>
       </c>
       <c r="E12" t="str">
         <v>owner7@sunrisevalley.com</v>
@@ -4301,7 +4301,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D13" t="str">
-        <v>Seema Menon</v>
+        <v>Usha Chauhan</v>
       </c>
       <c r="E13" t="str">
         <v>tenant1@sunrisevalley.com</v>
@@ -4336,7 +4336,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D14" t="str">
-        <v>Varun Iyer</v>
+        <v>Vinay Chauhan</v>
       </c>
       <c r="E14" t="str">
         <v>tenant2@sunrisevalley.com</v>
@@ -4371,7 +4371,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D15" t="str">
-        <v>Sangeeta Joshi</v>
+        <v>Priya Desai</v>
       </c>
       <c r="E15" t="str">
         <v>tenant3@sunrisevalley.com</v>
@@ -4406,7 +4406,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D16" t="str">
-        <v>Dev Pillai</v>
+        <v>Vikram Nair</v>
       </c>
       <c r="E16" t="str">
         <v>tenant4@sunrisevalley.com</v>
@@ -4441,7 +4441,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D17" t="str">
-        <v>Rajesh Choudhury</v>
+        <v>Usha Iyer</v>
       </c>
       <c r="E17" t="str">
         <v>tenant5@sunrisevalley.com</v>
@@ -4476,7 +4476,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D18" t="str">
-        <v>Simran Mehta</v>
+        <v>Shreya Reddy</v>
       </c>
       <c r="E18" t="str">
         <v>tenant6@sunrisevalley.com</v>
@@ -4511,7 +4511,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Yamini Menon</v>
+        <v>Bhavna Agarwal</v>
       </c>
       <c r="E19" t="str">
         <v>tenant7@sunrisevalley.com</v>
@@ -4546,7 +4546,7 @@
         <v>Family Member</v>
       </c>
       <c r="D20" t="str">
-        <v>Sanjay Joshi</v>
+        <v>Rohit Chauhan</v>
       </c>
       <c r="E20" t="str">
         <v>family1@sunrisevalley.com</v>
@@ -4581,7 +4581,7 @@
         <v>Family Member</v>
       </c>
       <c r="D21" t="str">
-        <v>Vishal Bhat</v>
+        <v>Bhavna Patel</v>
       </c>
       <c r="E21" t="str">
         <v>family2@sunrisevalley.com</v>
@@ -4662,7 +4662,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Lakshmi Ghosh</v>
+        <v>Aditi Rao</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@palmmeadows.com</v>
@@ -4697,7 +4697,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D3" t="str">
-        <v>Deepa Choudhury</v>
+        <v>Vinay Desai</v>
       </c>
       <c r="E3" t="str">
         <v>fm1@palmmeadows.com</v>
@@ -4732,7 +4732,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D4" t="str">
-        <v>Pooja Das</v>
+        <v>Rajesh Bose</v>
       </c>
       <c r="E4" t="str">
         <v>guard1@palmmeadows.com</v>
@@ -4767,7 +4767,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D5" t="str">
-        <v>Harish Bhat</v>
+        <v>Meera Nair</v>
       </c>
       <c r="E5" t="str">
         <v>owner1@palmmeadows.com</v>
@@ -4802,7 +4802,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D6" t="str">
-        <v>Sangeeta Pillai</v>
+        <v>Ananya Patel</v>
       </c>
       <c r="E6" t="str">
         <v>owner2@palmmeadows.com</v>
@@ -4837,7 +4837,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D7" t="str">
-        <v>Varun Joshi</v>
+        <v>Yamini Bose</v>
       </c>
       <c r="E7" t="str">
         <v>owner3@palmmeadows.com</v>
@@ -4872,7 +4872,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Ananya Bhat</v>
+        <v>Farhan Reddy</v>
       </c>
       <c r="E8" t="str">
         <v>owner4@palmmeadows.com</v>
@@ -4907,7 +4907,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Pooja Tiwari</v>
+        <v>Farhan Tiwari</v>
       </c>
       <c r="E9" t="str">
         <v>owner5@palmmeadows.com</v>
@@ -4942,7 +4942,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D10" t="str">
-        <v>Tanvi Nair</v>
+        <v>Vishal Jain</v>
       </c>
       <c r="E10" t="str">
         <v>tenant1@palmmeadows.com</v>
@@ -4977,7 +4977,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D11" t="str">
-        <v>Sneha Bose</v>
+        <v>Karan Iyer</v>
       </c>
       <c r="E11" t="str">
         <v>tenant2@palmmeadows.com</v>
@@ -5012,7 +5012,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D12" t="str">
-        <v>Shiv Mehta</v>
+        <v>Siddharth Verma</v>
       </c>
       <c r="E12" t="str">
         <v>tenant3@palmmeadows.com</v>
@@ -5047,7 +5047,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D13" t="str">
-        <v>Siddharth Joshi</v>
+        <v>Bhavna Bhat</v>
       </c>
       <c r="E13" t="str">
         <v>tenant4@palmmeadows.com</v>
@@ -5082,7 +5082,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D14" t="str">
-        <v>Akash Tiwari</v>
+        <v>Shiv Nair</v>
       </c>
       <c r="E14" t="str">
         <v>tenant5@palmmeadows.com</v>
@@ -5117,7 +5117,7 @@
         <v>Family Member</v>
       </c>
       <c r="D15" t="str">
-        <v>Tushar Desai</v>
+        <v>Arjun Patel</v>
       </c>
       <c r="E15" t="str">
         <v>family1@palmmeadows.com</v>
@@ -5152,7 +5152,7 @@
         <v>Family Member</v>
       </c>
       <c r="D16" t="str">
-        <v>Arjun Mehta</v>
+        <v>Pranav Kumar</v>
       </c>
       <c r="E16" t="str">
         <v>family2@palmmeadows.com</v>
@@ -5541,7 +5541,7 @@
         <v>Seed Execution Timestamp</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-08-20T09:13:54.920Z</v>
+        <v>2026-08-25T04:57:21.969Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement community notes, rbac engine, dynamic dashboard, and platform anti-lockout security
</commit_message>
<xml_diff>
--- a/Community_Testing_Credentials.xlsx
+++ b/Community_Testing_Credentials.xlsx
@@ -467,10 +467,10 @@
         <v>Super Admin</v>
       </c>
       <c r="E2" t="str">
-        <v>admin@managemygate.com</v>
+        <v>admin@enterprise.com</v>
       </c>
       <c r="F2" t="str">
-        <v>password123</v>
+        <v>SuperAdminPwd@123</v>
       </c>
       <c r="G2" t="str">
         <v>superadmin</v>
@@ -499,7 +499,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D3" t="str">
-        <v>Sapna Singh</v>
+        <v>Shiv Joshi</v>
       </c>
       <c r="E3" t="str">
         <v>admin1@greenfield.com</v>
@@ -534,7 +534,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D4" t="str">
-        <v>Shreya Bhat</v>
+        <v>Pranav Rao</v>
       </c>
       <c r="E4" t="str">
         <v>admin2@greenfield.com</v>
@@ -569,7 +569,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D5" t="str">
-        <v>Suresh Verma</v>
+        <v>Tushar Tiwari</v>
       </c>
       <c r="E5" t="str">
         <v>fm1@greenfield.com</v>
@@ -604,7 +604,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D6" t="str">
-        <v>Dev Tiwari</v>
+        <v>Seema Banerjee</v>
       </c>
       <c r="E6" t="str">
         <v>fm2@greenfield.com</v>
@@ -639,7 +639,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D7" t="str">
-        <v>Meera Sinha</v>
+        <v>Vinay Agarwal</v>
       </c>
       <c r="E7" t="str">
         <v>guard1@greenfield.com</v>
@@ -674,7 +674,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D8" t="str">
-        <v>Arjun Jain</v>
+        <v>Jaya Sinha</v>
       </c>
       <c r="E8" t="str">
         <v>guard2@greenfield.com</v>
@@ -709,7 +709,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Karan Rao</v>
+        <v>Harish Sharma</v>
       </c>
       <c r="E9" t="str">
         <v>owner1@greenfield.com</v>
@@ -744,7 +744,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Akash Joshi</v>
+        <v>Harish Ghosh</v>
       </c>
       <c r="E10" t="str">
         <v>owner2@greenfield.com</v>
@@ -779,7 +779,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Siddharth Sharma</v>
+        <v>Simran Pandey</v>
       </c>
       <c r="E11" t="str">
         <v>owner3@greenfield.com</v>
@@ -814,7 +814,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Ananya Pillai</v>
+        <v>Simran Gupta</v>
       </c>
       <c r="E12" t="str">
         <v>owner4@greenfield.com</v>
@@ -849,7 +849,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D13" t="str">
-        <v>Vinay Sharma</v>
+        <v>Neeraj Agarwal</v>
       </c>
       <c r="E13" t="str">
         <v>owner5@greenfield.com</v>
@@ -884,7 +884,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D14" t="str">
-        <v>Pranav Kapoor</v>
+        <v>Aditi Nair</v>
       </c>
       <c r="E14" t="str">
         <v>owner6@greenfield.com</v>
@@ -919,7 +919,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D15" t="str">
-        <v>Meera Iyer</v>
+        <v>Tushar Agarwal</v>
       </c>
       <c r="E15" t="str">
         <v>owner7@greenfield.com</v>
@@ -954,7 +954,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D16" t="str">
-        <v>Seema Menon</v>
+        <v>Neeraj Singh</v>
       </c>
       <c r="E16" t="str">
         <v>owner8@greenfield.com</v>
@@ -989,7 +989,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D17" t="str">
-        <v>Divya Pandey</v>
+        <v>Aditi Agarwal</v>
       </c>
       <c r="E17" t="str">
         <v>owner9@greenfield.com</v>
@@ -1024,7 +1024,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D18" t="str">
-        <v>Vinay Das</v>
+        <v>Jaya Choudhury</v>
       </c>
       <c r="E18" t="str">
         <v>owner10@greenfield.com</v>
@@ -1059,7 +1059,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Priya Reddy</v>
+        <v>Bhavna Tiwari</v>
       </c>
       <c r="E19" t="str">
         <v>tenant1@greenfield.com</v>
@@ -1094,7 +1094,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D20" t="str">
-        <v>Priya Mishra</v>
+        <v>Neeraj Sinha</v>
       </c>
       <c r="E20" t="str">
         <v>tenant2@greenfield.com</v>
@@ -1129,7 +1129,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D21" t="str">
-        <v>Ananya Pillai</v>
+        <v>Aditi Verma</v>
       </c>
       <c r="E21" t="str">
         <v>tenant3@greenfield.com</v>
@@ -1164,7 +1164,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D22" t="str">
-        <v>Shreya Chauhan</v>
+        <v>Usha Gupta</v>
       </c>
       <c r="E22" t="str">
         <v>tenant4@greenfield.com</v>
@@ -1199,7 +1199,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D23" t="str">
-        <v>Rekha Pandey</v>
+        <v>Nisha Pandey</v>
       </c>
       <c r="E23" t="str">
         <v>tenant5@greenfield.com</v>
@@ -1234,7 +1234,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D24" t="str">
-        <v>Priya Mehta</v>
+        <v>Siddharth Kumar</v>
       </c>
       <c r="E24" t="str">
         <v>tenant6@greenfield.com</v>
@@ -1269,7 +1269,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D25" t="str">
-        <v>Manav Jain</v>
+        <v>Shiv Joshi</v>
       </c>
       <c r="E25" t="str">
         <v>tenant7@greenfield.com</v>
@@ -1304,7 +1304,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D26" t="str">
-        <v>Sangeeta Pillai</v>
+        <v>Aditi Kumar</v>
       </c>
       <c r="E26" t="str">
         <v>tenant8@greenfield.com</v>
@@ -1339,7 +1339,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D27" t="str">
-        <v>Nisha Pandey</v>
+        <v>Sneha Reddy</v>
       </c>
       <c r="E27" t="str">
         <v>tenant9@greenfield.com</v>
@@ -1374,7 +1374,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D28" t="str">
-        <v>Karan Bhat</v>
+        <v>Dev Sinha</v>
       </c>
       <c r="E28" t="str">
         <v>tenant10@greenfield.com</v>
@@ -1409,7 +1409,7 @@
         <v>Family Member</v>
       </c>
       <c r="D29" t="str">
-        <v>Siddharth Mehta</v>
+        <v>Farhan Nair</v>
       </c>
       <c r="E29" t="str">
         <v>family1@greenfield.com</v>
@@ -1444,7 +1444,7 @@
         <v>Family Member</v>
       </c>
       <c r="D30" t="str">
-        <v>Tanvi Ghosh</v>
+        <v>Harish Shah</v>
       </c>
       <c r="E30" t="str">
         <v>family2@greenfield.com</v>
@@ -1479,7 +1479,7 @@
         <v>Family Member</v>
       </c>
       <c r="D31" t="str">
-        <v>Pranav Bose</v>
+        <v>Akash Shah</v>
       </c>
       <c r="E31" t="str">
         <v>family3@greenfield.com</v>
@@ -1514,7 +1514,7 @@
         <v>Family Member</v>
       </c>
       <c r="D32" t="str">
-        <v>Ananya Verma</v>
+        <v>Suresh Choudhury</v>
       </c>
       <c r="E32" t="str">
         <v>family4@greenfield.com</v>
@@ -1549,7 +1549,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D33" t="str">
-        <v>Aditi Bose</v>
+        <v>Gayatri Joshi</v>
       </c>
       <c r="E33" t="str">
         <v>admin1@sunrisevalley.com</v>
@@ -1584,7 +1584,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D34" t="str">
-        <v>Manav Pandey</v>
+        <v>Vinay Iyer</v>
       </c>
       <c r="E34" t="str">
         <v>fm1@sunrisevalley.com</v>
@@ -1619,7 +1619,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D35" t="str">
-        <v>Sangeeta Pandey</v>
+        <v>Vinay Agarwal</v>
       </c>
       <c r="E35" t="str">
         <v>guard1@sunrisevalley.com</v>
@@ -1654,7 +1654,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D36" t="str">
-        <v>Yamini Agarwal</v>
+        <v>Yamini Kapoor</v>
       </c>
       <c r="E36" t="str">
         <v>guard2@sunrisevalley.com</v>
@@ -1689,7 +1689,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D37" t="str">
-        <v>Dev Nair</v>
+        <v>Farhan Pandey</v>
       </c>
       <c r="E37" t="str">
         <v>owner1@sunrisevalley.com</v>
@@ -1724,7 +1724,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D38" t="str">
-        <v>Harish Rao</v>
+        <v>Siddharth Banerjee</v>
       </c>
       <c r="E38" t="str">
         <v>owner2@sunrisevalley.com</v>
@@ -1759,7 +1759,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D39" t="str">
-        <v>Ananya Desai</v>
+        <v>Rohit Gupta</v>
       </c>
       <c r="E39" t="str">
         <v>owner3@sunrisevalley.com</v>
@@ -1794,7 +1794,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D40" t="str">
-        <v>Zara Mehta</v>
+        <v>Zara Pillai</v>
       </c>
       <c r="E40" t="str">
         <v>owner4@sunrisevalley.com</v>
@@ -1829,7 +1829,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D41" t="str">
-        <v>Tanvi Joshi</v>
+        <v>Farhan Reddy</v>
       </c>
       <c r="E41" t="str">
         <v>owner5@sunrisevalley.com</v>
@@ -1864,7 +1864,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D42" t="str">
-        <v>Gayatri Kapoor</v>
+        <v>Sanjay Gupta</v>
       </c>
       <c r="E42" t="str">
         <v>owner6@sunrisevalley.com</v>
@@ -1899,7 +1899,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D43" t="str">
-        <v>Kavya Bhat</v>
+        <v>Sneha Ghosh</v>
       </c>
       <c r="E43" t="str">
         <v>owner7@sunrisevalley.com</v>
@@ -1934,7 +1934,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D44" t="str">
-        <v>Usha Chauhan</v>
+        <v>Siddharth Jain</v>
       </c>
       <c r="E44" t="str">
         <v>tenant1@sunrisevalley.com</v>
@@ -1969,7 +1969,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D45" t="str">
-        <v>Vinay Chauhan</v>
+        <v>Usha Desai</v>
       </c>
       <c r="E45" t="str">
         <v>tenant2@sunrisevalley.com</v>
@@ -2004,7 +2004,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D46" t="str">
-        <v>Priya Desai</v>
+        <v>Sanjay Mehta</v>
       </c>
       <c r="E46" t="str">
         <v>tenant3@sunrisevalley.com</v>
@@ -2039,7 +2039,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D47" t="str">
-        <v>Vikram Nair</v>
+        <v>Vishal Desai</v>
       </c>
       <c r="E47" t="str">
         <v>tenant4@sunrisevalley.com</v>
@@ -2074,7 +2074,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D48" t="str">
-        <v>Usha Iyer</v>
+        <v>Gayatri Kapoor</v>
       </c>
       <c r="E48" t="str">
         <v>tenant5@sunrisevalley.com</v>
@@ -2109,7 +2109,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D49" t="str">
-        <v>Shreya Reddy</v>
+        <v>Simran Jain</v>
       </c>
       <c r="E49" t="str">
         <v>tenant6@sunrisevalley.com</v>
@@ -2144,7 +2144,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D50" t="str">
-        <v>Bhavna Agarwal</v>
+        <v>Ishaan Iyer</v>
       </c>
       <c r="E50" t="str">
         <v>tenant7@sunrisevalley.com</v>
@@ -2179,7 +2179,7 @@
         <v>Family Member</v>
       </c>
       <c r="D51" t="str">
-        <v>Rohit Chauhan</v>
+        <v>Vishal Desai</v>
       </c>
       <c r="E51" t="str">
         <v>family1@sunrisevalley.com</v>
@@ -2214,7 +2214,7 @@
         <v>Family Member</v>
       </c>
       <c r="D52" t="str">
-        <v>Bhavna Patel</v>
+        <v>Rajesh Iyer</v>
       </c>
       <c r="E52" t="str">
         <v>family2@sunrisevalley.com</v>
@@ -2249,7 +2249,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D53" t="str">
-        <v>Aditi Rao</v>
+        <v>Dev Mishra</v>
       </c>
       <c r="E53" t="str">
         <v>admin1@palmmeadows.com</v>
@@ -2284,7 +2284,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D54" t="str">
-        <v>Vinay Desai</v>
+        <v>Aditi Bose</v>
       </c>
       <c r="E54" t="str">
         <v>fm1@palmmeadows.com</v>
@@ -2319,7 +2319,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D55" t="str">
-        <v>Rajesh Bose</v>
+        <v>Suresh Rao</v>
       </c>
       <c r="E55" t="str">
         <v>guard1@palmmeadows.com</v>
@@ -2354,7 +2354,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D56" t="str">
-        <v>Meera Nair</v>
+        <v>Shreya Kumar</v>
       </c>
       <c r="E56" t="str">
         <v>owner1@palmmeadows.com</v>
@@ -2389,7 +2389,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D57" t="str">
-        <v>Ananya Patel</v>
+        <v>Rajesh Reddy</v>
       </c>
       <c r="E57" t="str">
         <v>owner2@palmmeadows.com</v>
@@ -2424,7 +2424,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D58" t="str">
-        <v>Yamini Bose</v>
+        <v>Om Sinha</v>
       </c>
       <c r="E58" t="str">
         <v>owner3@palmmeadows.com</v>
@@ -2459,7 +2459,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D59" t="str">
-        <v>Farhan Reddy</v>
+        <v>Suresh Banerjee</v>
       </c>
       <c r="E59" t="str">
         <v>owner4@palmmeadows.com</v>
@@ -2494,7 +2494,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D60" t="str">
-        <v>Farhan Tiwari</v>
+        <v>Tanvi Pillai</v>
       </c>
       <c r="E60" t="str">
         <v>owner5@palmmeadows.com</v>
@@ -2529,7 +2529,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D61" t="str">
-        <v>Vishal Jain</v>
+        <v>Bhavna Singh</v>
       </c>
       <c r="E61" t="str">
         <v>tenant1@palmmeadows.com</v>
@@ -2564,7 +2564,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D62" t="str">
-        <v>Karan Iyer</v>
+        <v>Arjun Mehta</v>
       </c>
       <c r="E62" t="str">
         <v>tenant2@palmmeadows.com</v>
@@ -2599,7 +2599,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D63" t="str">
-        <v>Siddharth Verma</v>
+        <v>Pooja Verma</v>
       </c>
       <c r="E63" t="str">
         <v>tenant3@palmmeadows.com</v>
@@ -2634,7 +2634,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D64" t="str">
-        <v>Bhavna Bhat</v>
+        <v>Pranav Pandey</v>
       </c>
       <c r="E64" t="str">
         <v>tenant4@palmmeadows.com</v>
@@ -2669,7 +2669,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D65" t="str">
-        <v>Shiv Nair</v>
+        <v>Karan Chauhan</v>
       </c>
       <c r="E65" t="str">
         <v>tenant5@palmmeadows.com</v>
@@ -2704,7 +2704,7 @@
         <v>Family Member</v>
       </c>
       <c r="D66" t="str">
-        <v>Arjun Patel</v>
+        <v>Dev Banerjee</v>
       </c>
       <c r="E66" t="str">
         <v>family1@palmmeadows.com</v>
@@ -2739,7 +2739,7 @@
         <v>Family Member</v>
       </c>
       <c r="D67" t="str">
-        <v>Pranav Kumar</v>
+        <v>Seema Rao</v>
       </c>
       <c r="E67" t="str">
         <v>family2@palmmeadows.com</v>
@@ -2820,7 +2820,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Sapna Singh</v>
+        <v>Shiv Joshi</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@greenfield.com</v>
@@ -2855,7 +2855,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D3" t="str">
-        <v>Shreya Bhat</v>
+        <v>Pranav Rao</v>
       </c>
       <c r="E3" t="str">
         <v>admin2@greenfield.com</v>
@@ -2890,7 +2890,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D4" t="str">
-        <v>Suresh Verma</v>
+        <v>Tushar Tiwari</v>
       </c>
       <c r="E4" t="str">
         <v>fm1@greenfield.com</v>
@@ -2925,7 +2925,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D5" t="str">
-        <v>Dev Tiwari</v>
+        <v>Seema Banerjee</v>
       </c>
       <c r="E5" t="str">
         <v>fm2@greenfield.com</v>
@@ -2960,7 +2960,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D6" t="str">
-        <v>Meera Sinha</v>
+        <v>Vinay Agarwal</v>
       </c>
       <c r="E6" t="str">
         <v>guard1@greenfield.com</v>
@@ -2995,7 +2995,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D7" t="str">
-        <v>Arjun Jain</v>
+        <v>Jaya Sinha</v>
       </c>
       <c r="E7" t="str">
         <v>guard2@greenfield.com</v>
@@ -3030,7 +3030,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Karan Rao</v>
+        <v>Harish Sharma</v>
       </c>
       <c r="E8" t="str">
         <v>owner1@greenfield.com</v>
@@ -3065,7 +3065,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Akash Joshi</v>
+        <v>Harish Ghosh</v>
       </c>
       <c r="E9" t="str">
         <v>owner2@greenfield.com</v>
@@ -3100,7 +3100,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Siddharth Sharma</v>
+        <v>Simran Pandey</v>
       </c>
       <c r="E10" t="str">
         <v>owner3@greenfield.com</v>
@@ -3135,7 +3135,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Ananya Pillai</v>
+        <v>Simran Gupta</v>
       </c>
       <c r="E11" t="str">
         <v>owner4@greenfield.com</v>
@@ -3170,7 +3170,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Vinay Sharma</v>
+        <v>Neeraj Agarwal</v>
       </c>
       <c r="E12" t="str">
         <v>owner5@greenfield.com</v>
@@ -3205,7 +3205,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D13" t="str">
-        <v>Pranav Kapoor</v>
+        <v>Aditi Nair</v>
       </c>
       <c r="E13" t="str">
         <v>owner6@greenfield.com</v>
@@ -3240,7 +3240,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D14" t="str">
-        <v>Meera Iyer</v>
+        <v>Tushar Agarwal</v>
       </c>
       <c r="E14" t="str">
         <v>owner7@greenfield.com</v>
@@ -3275,7 +3275,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D15" t="str">
-        <v>Seema Menon</v>
+        <v>Neeraj Singh</v>
       </c>
       <c r="E15" t="str">
         <v>owner8@greenfield.com</v>
@@ -3310,7 +3310,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D16" t="str">
-        <v>Divya Pandey</v>
+        <v>Aditi Agarwal</v>
       </c>
       <c r="E16" t="str">
         <v>owner9@greenfield.com</v>
@@ -3345,7 +3345,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D17" t="str">
-        <v>Vinay Das</v>
+        <v>Jaya Choudhury</v>
       </c>
       <c r="E17" t="str">
         <v>owner10@greenfield.com</v>
@@ -3380,7 +3380,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D18" t="str">
-        <v>Priya Reddy</v>
+        <v>Bhavna Tiwari</v>
       </c>
       <c r="E18" t="str">
         <v>tenant1@greenfield.com</v>
@@ -3415,7 +3415,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Priya Mishra</v>
+        <v>Neeraj Sinha</v>
       </c>
       <c r="E19" t="str">
         <v>tenant2@greenfield.com</v>
@@ -3450,7 +3450,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D20" t="str">
-        <v>Ananya Pillai</v>
+        <v>Aditi Verma</v>
       </c>
       <c r="E20" t="str">
         <v>tenant3@greenfield.com</v>
@@ -3485,7 +3485,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D21" t="str">
-        <v>Shreya Chauhan</v>
+        <v>Usha Gupta</v>
       </c>
       <c r="E21" t="str">
         <v>tenant4@greenfield.com</v>
@@ -3520,7 +3520,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D22" t="str">
-        <v>Rekha Pandey</v>
+        <v>Nisha Pandey</v>
       </c>
       <c r="E22" t="str">
         <v>tenant5@greenfield.com</v>
@@ -3555,7 +3555,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D23" t="str">
-        <v>Priya Mehta</v>
+        <v>Siddharth Kumar</v>
       </c>
       <c r="E23" t="str">
         <v>tenant6@greenfield.com</v>
@@ -3590,7 +3590,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D24" t="str">
-        <v>Manav Jain</v>
+        <v>Shiv Joshi</v>
       </c>
       <c r="E24" t="str">
         <v>tenant7@greenfield.com</v>
@@ -3625,7 +3625,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D25" t="str">
-        <v>Sangeeta Pillai</v>
+        <v>Aditi Kumar</v>
       </c>
       <c r="E25" t="str">
         <v>tenant8@greenfield.com</v>
@@ -3660,7 +3660,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D26" t="str">
-        <v>Nisha Pandey</v>
+        <v>Sneha Reddy</v>
       </c>
       <c r="E26" t="str">
         <v>tenant9@greenfield.com</v>
@@ -3695,7 +3695,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D27" t="str">
-        <v>Karan Bhat</v>
+        <v>Dev Sinha</v>
       </c>
       <c r="E27" t="str">
         <v>tenant10@greenfield.com</v>
@@ -3730,7 +3730,7 @@
         <v>Family Member</v>
       </c>
       <c r="D28" t="str">
-        <v>Siddharth Mehta</v>
+        <v>Farhan Nair</v>
       </c>
       <c r="E28" t="str">
         <v>family1@greenfield.com</v>
@@ -3765,7 +3765,7 @@
         <v>Family Member</v>
       </c>
       <c r="D29" t="str">
-        <v>Tanvi Ghosh</v>
+        <v>Harish Shah</v>
       </c>
       <c r="E29" t="str">
         <v>family2@greenfield.com</v>
@@ -3800,7 +3800,7 @@
         <v>Family Member</v>
       </c>
       <c r="D30" t="str">
-        <v>Pranav Bose</v>
+        <v>Akash Shah</v>
       </c>
       <c r="E30" t="str">
         <v>family3@greenfield.com</v>
@@ -3835,7 +3835,7 @@
         <v>Family Member</v>
       </c>
       <c r="D31" t="str">
-        <v>Ananya Verma</v>
+        <v>Suresh Choudhury</v>
       </c>
       <c r="E31" t="str">
         <v>family4@greenfield.com</v>
@@ -3916,7 +3916,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Aditi Bose</v>
+        <v>Gayatri Joshi</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@sunrisevalley.com</v>
@@ -3951,7 +3951,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D3" t="str">
-        <v>Manav Pandey</v>
+        <v>Vinay Iyer</v>
       </c>
       <c r="E3" t="str">
         <v>fm1@sunrisevalley.com</v>
@@ -3986,7 +3986,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D4" t="str">
-        <v>Sangeeta Pandey</v>
+        <v>Vinay Agarwal</v>
       </c>
       <c r="E4" t="str">
         <v>guard1@sunrisevalley.com</v>
@@ -4021,7 +4021,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D5" t="str">
-        <v>Yamini Agarwal</v>
+        <v>Yamini Kapoor</v>
       </c>
       <c r="E5" t="str">
         <v>guard2@sunrisevalley.com</v>
@@ -4056,7 +4056,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D6" t="str">
-        <v>Dev Nair</v>
+        <v>Farhan Pandey</v>
       </c>
       <c r="E6" t="str">
         <v>owner1@sunrisevalley.com</v>
@@ -4091,7 +4091,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D7" t="str">
-        <v>Harish Rao</v>
+        <v>Siddharth Banerjee</v>
       </c>
       <c r="E7" t="str">
         <v>owner2@sunrisevalley.com</v>
@@ -4126,7 +4126,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Ananya Desai</v>
+        <v>Rohit Gupta</v>
       </c>
       <c r="E8" t="str">
         <v>owner3@sunrisevalley.com</v>
@@ -4161,7 +4161,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Zara Mehta</v>
+        <v>Zara Pillai</v>
       </c>
       <c r="E9" t="str">
         <v>owner4@sunrisevalley.com</v>
@@ -4196,7 +4196,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D10" t="str">
-        <v>Tanvi Joshi</v>
+        <v>Farhan Reddy</v>
       </c>
       <c r="E10" t="str">
         <v>owner5@sunrisevalley.com</v>
@@ -4231,7 +4231,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D11" t="str">
-        <v>Gayatri Kapoor</v>
+        <v>Sanjay Gupta</v>
       </c>
       <c r="E11" t="str">
         <v>owner6@sunrisevalley.com</v>
@@ -4266,7 +4266,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D12" t="str">
-        <v>Kavya Bhat</v>
+        <v>Sneha Ghosh</v>
       </c>
       <c r="E12" t="str">
         <v>owner7@sunrisevalley.com</v>
@@ -4301,7 +4301,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D13" t="str">
-        <v>Usha Chauhan</v>
+        <v>Siddharth Jain</v>
       </c>
       <c r="E13" t="str">
         <v>tenant1@sunrisevalley.com</v>
@@ -4336,7 +4336,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D14" t="str">
-        <v>Vinay Chauhan</v>
+        <v>Usha Desai</v>
       </c>
       <c r="E14" t="str">
         <v>tenant2@sunrisevalley.com</v>
@@ -4371,7 +4371,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D15" t="str">
-        <v>Priya Desai</v>
+        <v>Sanjay Mehta</v>
       </c>
       <c r="E15" t="str">
         <v>tenant3@sunrisevalley.com</v>
@@ -4406,7 +4406,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D16" t="str">
-        <v>Vikram Nair</v>
+        <v>Vishal Desai</v>
       </c>
       <c r="E16" t="str">
         <v>tenant4@sunrisevalley.com</v>
@@ -4441,7 +4441,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D17" t="str">
-        <v>Usha Iyer</v>
+        <v>Gayatri Kapoor</v>
       </c>
       <c r="E17" t="str">
         <v>tenant5@sunrisevalley.com</v>
@@ -4476,7 +4476,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D18" t="str">
-        <v>Shreya Reddy</v>
+        <v>Simran Jain</v>
       </c>
       <c r="E18" t="str">
         <v>tenant6@sunrisevalley.com</v>
@@ -4511,7 +4511,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D19" t="str">
-        <v>Bhavna Agarwal</v>
+        <v>Ishaan Iyer</v>
       </c>
       <c r="E19" t="str">
         <v>tenant7@sunrisevalley.com</v>
@@ -4546,7 +4546,7 @@
         <v>Family Member</v>
       </c>
       <c r="D20" t="str">
-        <v>Rohit Chauhan</v>
+        <v>Vishal Desai</v>
       </c>
       <c r="E20" t="str">
         <v>family1@sunrisevalley.com</v>
@@ -4581,7 +4581,7 @@
         <v>Family Member</v>
       </c>
       <c r="D21" t="str">
-        <v>Bhavna Patel</v>
+        <v>Rajesh Iyer</v>
       </c>
       <c r="E21" t="str">
         <v>family2@sunrisevalley.com</v>
@@ -4662,7 +4662,7 @@
         <v>Community Admin</v>
       </c>
       <c r="D2" t="str">
-        <v>Aditi Rao</v>
+        <v>Dev Mishra</v>
       </c>
       <c r="E2" t="str">
         <v>admin1@palmmeadows.com</v>
@@ -4697,7 +4697,7 @@
         <v>Facility Manager</v>
       </c>
       <c r="D3" t="str">
-        <v>Vinay Desai</v>
+        <v>Aditi Bose</v>
       </c>
       <c r="E3" t="str">
         <v>fm1@palmmeadows.com</v>
@@ -4732,7 +4732,7 @@
         <v>Security Guard</v>
       </c>
       <c r="D4" t="str">
-        <v>Rajesh Bose</v>
+        <v>Suresh Rao</v>
       </c>
       <c r="E4" t="str">
         <v>guard1@palmmeadows.com</v>
@@ -4767,7 +4767,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D5" t="str">
-        <v>Meera Nair</v>
+        <v>Shreya Kumar</v>
       </c>
       <c r="E5" t="str">
         <v>owner1@palmmeadows.com</v>
@@ -4802,7 +4802,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D6" t="str">
-        <v>Ananya Patel</v>
+        <v>Rajesh Reddy</v>
       </c>
       <c r="E6" t="str">
         <v>owner2@palmmeadows.com</v>
@@ -4837,7 +4837,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D7" t="str">
-        <v>Yamini Bose</v>
+        <v>Om Sinha</v>
       </c>
       <c r="E7" t="str">
         <v>owner3@palmmeadows.com</v>
@@ -4872,7 +4872,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D8" t="str">
-        <v>Farhan Reddy</v>
+        <v>Suresh Banerjee</v>
       </c>
       <c r="E8" t="str">
         <v>owner4@palmmeadows.com</v>
@@ -4907,7 +4907,7 @@
         <v>Resident Owner</v>
       </c>
       <c r="D9" t="str">
-        <v>Farhan Tiwari</v>
+        <v>Tanvi Pillai</v>
       </c>
       <c r="E9" t="str">
         <v>owner5@palmmeadows.com</v>
@@ -4942,7 +4942,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D10" t="str">
-        <v>Vishal Jain</v>
+        <v>Bhavna Singh</v>
       </c>
       <c r="E10" t="str">
         <v>tenant1@palmmeadows.com</v>
@@ -4977,7 +4977,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D11" t="str">
-        <v>Karan Iyer</v>
+        <v>Arjun Mehta</v>
       </c>
       <c r="E11" t="str">
         <v>tenant2@palmmeadows.com</v>
@@ -5012,7 +5012,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D12" t="str">
-        <v>Siddharth Verma</v>
+        <v>Pooja Verma</v>
       </c>
       <c r="E12" t="str">
         <v>tenant3@palmmeadows.com</v>
@@ -5047,7 +5047,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D13" t="str">
-        <v>Bhavna Bhat</v>
+        <v>Pranav Pandey</v>
       </c>
       <c r="E13" t="str">
         <v>tenant4@palmmeadows.com</v>
@@ -5082,7 +5082,7 @@
         <v>Resident Tenant</v>
       </c>
       <c r="D14" t="str">
-        <v>Shiv Nair</v>
+        <v>Karan Chauhan</v>
       </c>
       <c r="E14" t="str">
         <v>tenant5@palmmeadows.com</v>
@@ -5117,7 +5117,7 @@
         <v>Family Member</v>
       </c>
       <c r="D15" t="str">
-        <v>Arjun Patel</v>
+        <v>Dev Banerjee</v>
       </c>
       <c r="E15" t="str">
         <v>family1@palmmeadows.com</v>
@@ -5152,7 +5152,7 @@
         <v>Family Member</v>
       </c>
       <c r="D16" t="str">
-        <v>Pranav Kumar</v>
+        <v>Seema Rao</v>
       </c>
       <c r="E16" t="str">
         <v>family2@palmmeadows.com</v>
@@ -5322,7 +5322,7 @@
         <v>Platform Multi-Community Switch</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Login with admin@managemygate.com / password123.
+        <v xml:space="preserve">1. Login with admin@enterprise.com / SuperAdminPwd@123.
 2. Open workspace dropdown in header.
 3. Verify all 3 communities (Greenfield Heights, Sunrise Valley, Palm Meadows) are listed.
 4. Switch workspace and verify context changes.</v>
@@ -5517,7 +5517,7 @@
         <v>Super Admin Account</v>
       </c>
       <c r="B7" t="str">
-        <v>admin@managemygate.com (Password: password123)</v>
+        <v>admin@enterprise.com (Password: SuperAdminPwd@123)</v>
       </c>
     </row>
     <row r="8">
@@ -5541,7 +5541,7 @@
         <v>Seed Execution Timestamp</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-08-25T04:57:21.969Z</v>
+        <v>2026-08-31T11:04:51.348Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>